<commit_message>
implemented and validated the missing remakrs issue and scheduled normalization and detection has been standardized
</commit_message>
<xml_diff>
--- a/output/DTR_7-4_.BELBES_M.xlsx
+++ b/output/DTR_7-4_.BELBES_M.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
   <si>
     <t>Republic of the Philippines</t>
   </si>
@@ -74,6 +74,18 @@
   </si>
   <si>
     <t>Minutes</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Eid'l Fitr</t>
+  </si>
+  <si>
+    <t>Sunday / Palm Sunday</t>
   </si>
   <si>
     <t>Total</t>
@@ -879,14 +891,16 @@
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
-      <c r="H19" s="23"/>
+      <c r="H19" s="23" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="20" spans="1:11" s="7" customFormat="1">
       <c r="A20" s="22">
         <v>2</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
@@ -898,7 +912,7 @@
         <v>3</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
@@ -910,7 +924,7 @@
         <v>4</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
@@ -922,7 +936,7 @@
         <v>5</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
@@ -934,7 +948,7 @@
         <v>6</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
@@ -949,7 +963,9 @@
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
-      <c r="H25" s="23"/>
+      <c r="H25" s="23" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="26" spans="1:11" s="7" customFormat="1">
       <c r="A26" s="21">
@@ -959,14 +975,16 @@
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
-      <c r="H26" s="23"/>
+      <c r="H26" s="23" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="27" spans="1:11" s="7" customFormat="1">
       <c r="A27" s="22">
         <v>9</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
@@ -978,7 +996,7 @@
         <v>10</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
@@ -990,7 +1008,7 @@
         <v>11</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
@@ -1002,7 +1020,7 @@
         <v>12</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
@@ -1014,7 +1032,7 @@
         <v>13</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -1029,7 +1047,9 @@
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
-      <c r="H32" s="23"/>
+      <c r="H32" s="23" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="33" spans="1:11" s="7" customFormat="1">
       <c r="A33" s="21">
@@ -1039,14 +1059,16 @@
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
-      <c r="H33" s="23"/>
+      <c r="H33" s="23" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="34" spans="1:11" s="7" customFormat="1">
       <c r="A34" s="22">
         <v>16</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
@@ -1058,7 +1080,7 @@
         <v>17</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
@@ -1070,7 +1092,7 @@
         <v>18</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -1082,7 +1104,7 @@
         <v>19</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
@@ -1097,7 +1119,9 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
-      <c r="H38" s="23"/>
+      <c r="H38" s="23" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="39" spans="1:11" s="8" customFormat="1">
       <c r="A39" s="21">
@@ -1107,7 +1131,9 @@
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
       <c r="E39" s="8"/>
-      <c r="H39" s="23"/>
+      <c r="H39" s="23" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="40" spans="1:11" s="7" customFormat="1">
       <c r="A40" s="21">
@@ -1117,7 +1143,9 @@
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
       <c r="E40" s="7"/>
-      <c r="H40" s="23"/>
+      <c r="H40" s="23" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="41" spans="1:11" s="7" customFormat="1">
       <c r="A41" s="22">
@@ -1144,7 +1172,7 @@
         <v>25</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
@@ -1156,7 +1184,7 @@
         <v>26</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -1168,7 +1196,7 @@
         <v>27</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
@@ -1183,7 +1211,9 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
-      <c r="H46" s="23"/>
+      <c r="H46" s="23" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="47" spans="1:11" s="7" customFormat="1">
       <c r="A47" s="21">
@@ -1193,14 +1223,16 @@
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
-      <c r="H47" s="23"/>
+      <c r="H47" s="23" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="48" spans="1:11" s="7" customFormat="1">
       <c r="A48" s="24">
         <v>30</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
@@ -1212,7 +1244,7 @@
         <v>31</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
@@ -1221,7 +1253,7 @@
     </row>
     <row r="50" spans="1:11" s="7" customFormat="1">
       <c r="A50" s="25" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G50" s="26" t="str">
         <f>SUM(G20:G49)</f>
@@ -1232,12 +1264,12 @@
     <row r="51" spans="1:11" s="7" customFormat="1"/>
     <row r="52" spans="1:11" s="7" customFormat="1">
       <c r="A52" s="27" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="53" spans="1:11" s="7" customFormat="1">
       <c r="A53" s="7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="54" spans="1:11" customHeight="1" ht="15" s="7" customFormat="1"/>
@@ -1248,29 +1280,29 @@
     </row>
     <row r="56" spans="1:11" s="7" customFormat="1">
       <c r="A56" s="29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:11" s="7" customFormat="1"/>
     <row r="58" spans="1:11" s="7" customFormat="1">
       <c r="A58" s="30" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="59" spans="1:11" s="7" customFormat="1">
       <c r="B59" s="31" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:11" s="7" customFormat="1"/>
     <row r="61" spans="1:11" s="7" customFormat="1">
       <c r="A61" s="32" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="62" spans="1:11" s="7" customFormat="1">
       <c r="A62" s="16" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="63" spans="1:11" customHeight="1" ht="15" s="7" customFormat="1"/>
@@ -1361,47 +1393,47 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(dtr): restore missing generated time data for AM/PM two-row raw headers
</commit_message>
<xml_diff>
--- a/output/DTR_7-4_.BELBES_M.xlsx
+++ b/output/DTR_7-4_.BELBES_M.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="75">
   <si>
     <t>Republic of the Philippines</t>
   </si>
@@ -115,52 +115,109 @@
     <t>06:44</t>
   </si>
   <si>
+    <t>16:43</t>
+  </si>
+  <si>
     <t>06:49</t>
   </si>
   <si>
+    <t>16:01</t>
+  </si>
+  <si>
     <t>06:47</t>
   </si>
   <si>
+    <t>16:15</t>
+  </si>
+  <si>
     <t>06:34</t>
   </si>
   <si>
+    <t>15:19</t>
+  </si>
+  <si>
     <t>06:40</t>
   </si>
   <si>
+    <t>14:47</t>
+  </si>
+  <si>
     <t>06:31</t>
   </si>
   <si>
+    <t>16:03</t>
+  </si>
+  <si>
     <t>06:37</t>
   </si>
   <si>
+    <t>15:29</t>
+  </si>
+  <si>
     <t>06:36</t>
   </si>
   <si>
+    <t>15:26</t>
+  </si>
+  <si>
     <t>07:13</t>
   </si>
   <si>
+    <t>16:04</t>
+  </si>
+  <si>
+    <t>15:50</t>
+  </si>
+  <si>
     <t>06:11</t>
   </si>
   <si>
+    <t>15:44</t>
+  </si>
+  <si>
     <t>06:30</t>
   </si>
   <si>
+    <t>15:48</t>
+  </si>
+  <si>
     <t>06:51</t>
   </si>
   <si>
+    <t>16:10</t>
+  </si>
+  <si>
     <t>08:14</t>
   </si>
   <si>
+    <t>15:07</t>
+  </si>
+  <si>
     <t>07:05</t>
   </si>
   <si>
+    <t>16:37</t>
+  </si>
+  <si>
     <t>07:58</t>
   </si>
   <si>
+    <t>16:16</t>
+  </si>
+  <si>
+    <t>12:46</t>
+  </si>
+  <si>
     <t>06:41</t>
   </si>
   <si>
+    <t>16:28</t>
+  </si>
+  <si>
     <t>06:58</t>
+  </si>
+  <si>
+    <t>17:12</t>
   </si>
   <si>
     <t>on Forced/Mandatory Leave</t>
@@ -904,7 +961,9 @@
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
+      <c r="E20" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:11" s="7" customFormat="1">
@@ -912,11 +971,13 @@
         <v>3</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
+      <c r="E21" s="7" t="s">
+        <v>33</v>
+      </c>
       <c r="H21" s="7"/>
     </row>
     <row r="22" spans="1:11" s="8" customFormat="1">
@@ -924,11 +985,13 @@
         <v>4</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
+      <c r="E22" s="8" t="s">
+        <v>35</v>
+      </c>
       <c r="H22" s="8"/>
     </row>
     <row r="23" spans="1:11" s="7" customFormat="1">
@@ -936,11 +999,13 @@
         <v>5</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
+      <c r="E23" s="7" t="s">
+        <v>37</v>
+      </c>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:11" s="7" customFormat="1">
@@ -948,11 +1013,13 @@
         <v>6</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
+      <c r="E24" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:11" s="7" customFormat="1">
@@ -984,11 +1051,13 @@
         <v>9</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
+      <c r="E27" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="H27" s="7"/>
     </row>
     <row r="28" spans="1:11" s="7" customFormat="1">
@@ -996,11 +1065,13 @@
         <v>10</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
+      <c r="E28" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="1:11" s="7" customFormat="1">
@@ -1008,11 +1079,13 @@
         <v>11</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
+      <c r="E29" s="7" t="s">
+        <v>45</v>
+      </c>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="1:11" s="7" customFormat="1">
@@ -1020,11 +1093,13 @@
         <v>12</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
+      <c r="E30" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:11" s="7" customFormat="1">
@@ -1036,7 +1111,9 @@
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
+      <c r="E31" s="7" t="s">
+        <v>48</v>
+      </c>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:11" s="7" customFormat="1">
@@ -1068,11 +1145,13 @@
         <v>16</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
+      <c r="E34" s="7" t="s">
+        <v>50</v>
+      </c>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:11" s="7" customFormat="1">
@@ -1080,11 +1159,13 @@
         <v>17</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
+      <c r="E35" s="7" t="s">
+        <v>52</v>
+      </c>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:11" s="7" customFormat="1">
@@ -1092,11 +1173,13 @@
         <v>18</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
+      <c r="E36" s="7" t="s">
+        <v>54</v>
+      </c>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="1:11" s="7" customFormat="1">
@@ -1104,11 +1187,13 @@
         <v>19</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
+      <c r="E37" s="7" t="s">
+        <v>56</v>
+      </c>
       <c r="H37" s="7"/>
     </row>
     <row r="38" spans="1:11" s="7" customFormat="1">
@@ -1172,11 +1257,13 @@
         <v>25</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
+      <c r="E43" s="8" t="s">
+        <v>58</v>
+      </c>
       <c r="H43" s="8"/>
     </row>
     <row r="44" spans="1:11" s="8" customFormat="1">
@@ -1184,11 +1271,13 @@
         <v>26</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
+      <c r="E44" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="H44" s="8"/>
     </row>
     <row r="45" spans="1:11" s="7" customFormat="1">
@@ -1196,11 +1285,13 @@
         <v>27</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
-      <c r="E45" s="7"/>
+      <c r="E45" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:11" s="7" customFormat="1">
@@ -1232,11 +1323,13 @@
         <v>30</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
-      <c r="E48" s="7"/>
+      <c r="E48" s="7" t="s">
+        <v>63</v>
+      </c>
       <c r="H48" s="7"/>
     </row>
     <row r="49" spans="1:11" s="7" customFormat="1">
@@ -1244,11 +1337,13 @@
         <v>31</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
-      <c r="E49" s="7"/>
+      <c r="E49" s="7" t="s">
+        <v>65</v>
+      </c>
       <c r="H49" s="7"/>
     </row>
     <row r="50" spans="1:11" s="7" customFormat="1">
@@ -1393,47 +1488,47 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="3" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="4" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="3" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>